<commit_message>
docs: add Fixed Assets & Revaluation to user guide + UAT tracker
- Word: new section 13 (Fixed Assets, Depreciation & Revaluation) with
  feature list, user guide and AS-01..AS-06 test scenarios; module count
  updated to 12; End-to-End renumbered to 14.
- UAT tracker: +6 cases (AS-01..AS-06), total 49; Summary auto-includes
  the Fixed Assets module.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016VgZWku95cicE6VZPkFTLL
</commit_message>
<xml_diff>
--- a/docs/UAT_Tracker_Custom_Modules.xlsx
+++ b/docs/UAT_Tracker_Custom_Modules.xlsx
@@ -530,7 +530,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J44"/>
+  <dimension ref="A1:J50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2120,27 +2120,27 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>E2E-1</t>
+          <t>AS-01</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>End-to-End</t>
+          <t>Fixed Assets</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Onboarding tenant</t>
+          <t>Board garis lurus</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Lead → Create Lease Contract → aktifkan → Handover Move-in → Guarantee.</t>
+          <t>Aset 10jt, salvage 0, linear, jumlah=5, periode=12. Compute Depreciation.</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>Kontrak aktif; handover selesai; jaminan Active; tenant bisa login portal.</t>
+          <t>5 baris @ 2jt; akumulasi akhir=10jt; remaining akhir=0.</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -2160,27 +2160,27 @@
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>E2E-2</t>
+          <t>AS-02</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>End-to-End</t>
+          <t>Fixed Assets</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>Billing bulanan</t>
+          <t>Posting penyusutan</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>Invoice sewa + Meter recharge + GTO turnover diposting.</t>
+          <t>Confirm; tanggal baris ≤ hari ini; Post Due Depreciation.</t>
         </is>
       </c>
       <c r="E41" s="7" t="inlineStr">
         <is>
-          <t>Semua pendapatan ber-link properti &amp; analytic; muncul di Owners Statement.</t>
+          <t>Jurnal Dr Beban/Cr Akumulasi posted; ber-tag properti (analytic).</t>
         </is>
       </c>
       <c r="F41" s="5" t="inlineStr">
@@ -2200,32 +2200,32 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>E2E-3</t>
+          <t>AS-03</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>End-to-End</t>
+          <t>Fixed Assets</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Pengeluaran</t>
+          <t>Saldo menurun</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Maintenance → Create PO → terima → vendor bill posted.</t>
+          <t>Aset declining, factor=2, jumlah=5. Compute.</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>Beban masuk Payment Details &amp; analytic properti.</t>
+          <t>Nominal menurun tiap periode; baris terakhir menutup ke salvage.</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -2240,27 +2240,27 @@
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>E2E-4</t>
+          <t>AS-04</t>
         </is>
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>End-to-End</t>
+          <t>Fixed Assets</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>Tutup periode</t>
+          <t>Revaluation naik</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>Cetak Owners Statement; Owner Remittance; ekspor CORETAX Faktur PK.</t>
+          <t>Tambah revaluation +5jt → Post Revaluations.</t>
         </is>
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t>Laporan konsisten; remittance terposting; XML e-Faktur terunduh.</t>
+          <t>Jurnal Dr Aset/Cr Reserve 5jt; gross naik; board recompute.</t>
         </is>
       </c>
       <c r="F43" s="5" t="inlineStr">
@@ -2280,27 +2280,27 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>E2E-5</t>
+          <t>AS-05</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>End-to-End</t>
+          <t>Fixed Assets</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Move-out</t>
+          <t>Revaluation turun</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Handover Move-out + make-good; Security Deposit refund; kontrak ditutup.</t>
+          <t>Tambah revaluation −2jt → Post Revaluations.</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>Deposit terselesaikan; Sec Dep Bal nol; kontrak closed.</t>
+          <t>Jurnal Dr Reserve/Cr Aset 2jt; gross turun; board recompute.</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -2317,9 +2317,249 @@
       <c r="I44" s="2" t="inlineStr"/>
       <c r="J44" s="4" t="inlineStr"/>
     </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>AS-06</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>Fixed Assets</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>Sync CORETAX L9</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>Klik Sync CORETAX L9 (coretax terpasang).</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="inlineStr">
+        <is>
+          <t>Entri coretax.asset.depreciation terbuat dgn nilai perolehan &amp; penyusutan tahun berjalan.</t>
+        </is>
+      </c>
+      <c r="F45" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G45" s="5" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="H45" s="6" t="inlineStr"/>
+      <c r="I45" s="5" t="inlineStr"/>
+      <c r="J45" s="7" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>E2E-1</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>End-to-End</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>Onboarding tenant</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>Lead → Create Lease Contract → aktifkan → Handover Move-in → Guarantee.</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t>Kontrak aktif; handover selesai; jaminan Active; tenant bisa login portal.</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="inlineStr"/>
+      <c r="I46" s="2" t="inlineStr"/>
+      <c r="J46" s="4" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>E2E-2</t>
+        </is>
+      </c>
+      <c r="B47" s="6" t="inlineStr">
+        <is>
+          <t>End-to-End</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>Billing bulanan</t>
+        </is>
+      </c>
+      <c r="D47" s="7" t="inlineStr">
+        <is>
+          <t>Invoice sewa + Meter recharge + GTO turnover diposting.</t>
+        </is>
+      </c>
+      <c r="E47" s="7" t="inlineStr">
+        <is>
+          <t>Semua pendapatan ber-link properti &amp; analytic; muncul di Owners Statement.</t>
+        </is>
+      </c>
+      <c r="F47" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G47" s="5" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="H47" s="6" t="inlineStr"/>
+      <c r="I47" s="5" t="inlineStr"/>
+      <c r="J47" s="7" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>E2E-3</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>End-to-End</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>Pengeluaran</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>Maintenance → Create PO → terima → vendor bill posted.</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="inlineStr">
+        <is>
+          <t>Beban masuk Payment Details &amp; analytic properti.</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr"/>
+      <c r="I48" s="2" t="inlineStr"/>
+      <c r="J48" s="4" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>E2E-4</t>
+        </is>
+      </c>
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>End-to-End</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="inlineStr">
+        <is>
+          <t>Tutup periode</t>
+        </is>
+      </c>
+      <c r="D49" s="7" t="inlineStr">
+        <is>
+          <t>Cetak Owners Statement; Owner Remittance; ekspor CORETAX Faktur PK.</t>
+        </is>
+      </c>
+      <c r="E49" s="7" t="inlineStr">
+        <is>
+          <t>Laporan konsisten; remittance terposting; XML e-Faktur terunduh.</t>
+        </is>
+      </c>
+      <c r="F49" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G49" s="5" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="H49" s="6" t="inlineStr"/>
+      <c r="I49" s="5" t="inlineStr"/>
+      <c r="J49" s="7" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>E2E-5</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>End-to-End</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>Move-out</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>Handover Move-out + make-good; Security Deposit refund; kontrak ditutup.</t>
+        </is>
+      </c>
+      <c r="E50" s="4" t="inlineStr">
+        <is>
+          <t>Deposit terselesaikan; Sec Dep Bal nol; kontrak closed.</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="H50" s="3" t="inlineStr"/>
+      <c r="I50" s="2" t="inlineStr"/>
+      <c r="J50" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
-  <conditionalFormatting sqref="G2:G44">
+  <conditionalFormatting sqref="G2:G50">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -2334,10 +2574,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="G2:G44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G2:G50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not Run,Pass,Fail,Blocked,N/A"</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"High,Medium,Low"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2351,7 +2591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2375,7 +2615,7 @@
         </is>
       </c>
       <c r="B3" s="10">
-        <f>COUNTA('Test Cases'!A2:A44)</f>
+        <f>COUNTA('Test Cases'!A2:A50)</f>
         <v/>
       </c>
     </row>
@@ -2386,7 +2626,7 @@
         </is>
       </c>
       <c r="B4" s="10">
-        <f>COUNTIF('Test Cases'!G2:G44,"Pass")</f>
+        <f>COUNTIF('Test Cases'!G2:G50,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -2397,7 +2637,7 @@
         </is>
       </c>
       <c r="B5" s="10">
-        <f>COUNTIF('Test Cases'!G2:G44,"Fail")</f>
+        <f>COUNTIF('Test Cases'!G2:G50,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -2408,7 +2648,7 @@
         </is>
       </c>
       <c r="B6" s="10">
-        <f>COUNTIF('Test Cases'!G2:G44,"Blocked")</f>
+        <f>COUNTIF('Test Cases'!G2:G50,"Blocked")</f>
         <v/>
       </c>
     </row>
@@ -2419,7 +2659,7 @@
         </is>
       </c>
       <c r="B7" s="10">
-        <f>COUNTIF('Test Cases'!G2:G44,"N/A")</f>
+        <f>COUNTIF('Test Cases'!G2:G50,"N/A")</f>
         <v/>
       </c>
     </row>
@@ -2430,7 +2670,7 @@
         </is>
       </c>
       <c r="B8" s="10">
-        <f>COUNTIF('Test Cases'!G2:G44,"Not Run")</f>
+        <f>COUNTIF('Test Cases'!G2:G50,"Not Run")</f>
         <v/>
       </c>
     </row>
@@ -2486,19 +2726,19 @@
         </is>
       </c>
       <c r="B13" s="10">
-        <f>COUNTIF('Test Cases'!B2:B44,A13)</f>
+        <f>COUNTIF('Test Cases'!B2:B50,A13)</f>
         <v/>
       </c>
       <c r="C13" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B44,A13,'Test Cases'!G2:G44,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!B2:B50,A13,'Test Cases'!G2:G50,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B44,A13,'Test Cases'!G2:G44,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!B2:B50,A13,'Test Cases'!G2:G50,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B44,A13,'Test Cases'!G2:G44,"Not Run")</f>
+        <f>COUNTIFS('Test Cases'!B2:B50,A13,'Test Cases'!G2:G50,"Not Run")</f>
         <v/>
       </c>
     </row>
@@ -2509,19 +2749,19 @@
         </is>
       </c>
       <c r="B14" s="10">
-        <f>COUNTIF('Test Cases'!B2:B44,A14)</f>
+        <f>COUNTIF('Test Cases'!B2:B50,A14)</f>
         <v/>
       </c>
       <c r="C14" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B44,A14,'Test Cases'!G2:G44,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!B2:B50,A14,'Test Cases'!G2:G50,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B44,A14,'Test Cases'!G2:G44,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!B2:B50,A14,'Test Cases'!G2:G50,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B44,A14,'Test Cases'!G2:G44,"Not Run")</f>
+        <f>COUNTIFS('Test Cases'!B2:B50,A14,'Test Cases'!G2:G50,"Not Run")</f>
         <v/>
       </c>
     </row>
@@ -2532,19 +2772,19 @@
         </is>
       </c>
       <c r="B15" s="10">
-        <f>COUNTIF('Test Cases'!B2:B44,A15)</f>
+        <f>COUNTIF('Test Cases'!B2:B50,A15)</f>
         <v/>
       </c>
       <c r="C15" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B44,A15,'Test Cases'!G2:G44,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!B2:B50,A15,'Test Cases'!G2:G50,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B44,A15,'Test Cases'!G2:G44,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!B2:B50,A15,'Test Cases'!G2:G50,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B44,A15,'Test Cases'!G2:G44,"Not Run")</f>
+        <f>COUNTIFS('Test Cases'!B2:B50,A15,'Test Cases'!G2:G50,"Not Run")</f>
         <v/>
       </c>
     </row>
@@ -2555,19 +2795,19 @@
         </is>
       </c>
       <c r="B16" s="10">
-        <f>COUNTIF('Test Cases'!B2:B44,A16)</f>
+        <f>COUNTIF('Test Cases'!B2:B50,A16)</f>
         <v/>
       </c>
       <c r="C16" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B44,A16,'Test Cases'!G2:G44,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!B2:B50,A16,'Test Cases'!G2:G50,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B44,A16,'Test Cases'!G2:G44,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!B2:B50,A16,'Test Cases'!G2:G50,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B44,A16,'Test Cases'!G2:G44,"Not Run")</f>
+        <f>COUNTIFS('Test Cases'!B2:B50,A16,'Test Cases'!G2:G50,"Not Run")</f>
         <v/>
       </c>
     </row>
@@ -2578,19 +2818,19 @@
         </is>
       </c>
       <c r="B17" s="10">
-        <f>COUNTIF('Test Cases'!B2:B44,A17)</f>
+        <f>COUNTIF('Test Cases'!B2:B50,A17)</f>
         <v/>
       </c>
       <c r="C17" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B44,A17,'Test Cases'!G2:G44,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!B2:B50,A17,'Test Cases'!G2:G50,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B44,A17,'Test Cases'!G2:G44,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!B2:B50,A17,'Test Cases'!G2:G50,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B44,A17,'Test Cases'!G2:G44,"Not Run")</f>
+        <f>COUNTIFS('Test Cases'!B2:B50,A17,'Test Cases'!G2:G50,"Not Run")</f>
         <v/>
       </c>
     </row>
@@ -2601,19 +2841,19 @@
         </is>
       </c>
       <c r="B18" s="10">
-        <f>COUNTIF('Test Cases'!B2:B44,A18)</f>
+        <f>COUNTIF('Test Cases'!B2:B50,A18)</f>
         <v/>
       </c>
       <c r="C18" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B44,A18,'Test Cases'!G2:G44,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!B2:B50,A18,'Test Cases'!G2:G50,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B44,A18,'Test Cases'!G2:G44,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!B2:B50,A18,'Test Cases'!G2:G50,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B44,A18,'Test Cases'!G2:G44,"Not Run")</f>
+        <f>COUNTIFS('Test Cases'!B2:B50,A18,'Test Cases'!G2:G50,"Not Run")</f>
         <v/>
       </c>
     </row>
@@ -2624,19 +2864,19 @@
         </is>
       </c>
       <c r="B19" s="10">
-        <f>COUNTIF('Test Cases'!B2:B44,A19)</f>
+        <f>COUNTIF('Test Cases'!B2:B50,A19)</f>
         <v/>
       </c>
       <c r="C19" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B44,A19,'Test Cases'!G2:G44,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!B2:B50,A19,'Test Cases'!G2:G50,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B44,A19,'Test Cases'!G2:G44,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!B2:B50,A19,'Test Cases'!G2:G50,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B44,A19,'Test Cases'!G2:G44,"Not Run")</f>
+        <f>COUNTIFS('Test Cases'!B2:B50,A19,'Test Cases'!G2:G50,"Not Run")</f>
         <v/>
       </c>
     </row>
@@ -2647,19 +2887,19 @@
         </is>
       </c>
       <c r="B20" s="10">
-        <f>COUNTIF('Test Cases'!B2:B44,A20)</f>
+        <f>COUNTIF('Test Cases'!B2:B50,A20)</f>
         <v/>
       </c>
       <c r="C20" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B44,A20,'Test Cases'!G2:G44,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!B2:B50,A20,'Test Cases'!G2:G50,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B44,A20,'Test Cases'!G2:G44,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!B2:B50,A20,'Test Cases'!G2:G50,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B44,A20,'Test Cases'!G2:G44,"Not Run")</f>
+        <f>COUNTIFS('Test Cases'!B2:B50,A20,'Test Cases'!G2:G50,"Not Run")</f>
         <v/>
       </c>
     </row>
@@ -2670,19 +2910,19 @@
         </is>
       </c>
       <c r="B21" s="10">
-        <f>COUNTIF('Test Cases'!B2:B44,A21)</f>
+        <f>COUNTIF('Test Cases'!B2:B50,A21)</f>
         <v/>
       </c>
       <c r="C21" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B44,A21,'Test Cases'!G2:G44,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!B2:B50,A21,'Test Cases'!G2:G50,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B44,A21,'Test Cases'!G2:G44,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!B2:B50,A21,'Test Cases'!G2:G50,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B44,A21,'Test Cases'!G2:G44,"Not Run")</f>
+        <f>COUNTIFS('Test Cases'!B2:B50,A21,'Test Cases'!G2:G50,"Not Run")</f>
         <v/>
       </c>
     </row>
@@ -2693,19 +2933,19 @@
         </is>
       </c>
       <c r="B22" s="10">
-        <f>COUNTIF('Test Cases'!B2:B44,A22)</f>
+        <f>COUNTIF('Test Cases'!B2:B50,A22)</f>
         <v/>
       </c>
       <c r="C22" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B44,A22,'Test Cases'!G2:G44,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!B2:B50,A22,'Test Cases'!G2:G50,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B44,A22,'Test Cases'!G2:G44,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!B2:B50,A22,'Test Cases'!G2:G50,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B44,A22,'Test Cases'!G2:G44,"Not Run")</f>
+        <f>COUNTIFS('Test Cases'!B2:B50,A22,'Test Cases'!G2:G50,"Not Run")</f>
         <v/>
       </c>
     </row>
@@ -2716,42 +2956,65 @@
         </is>
       </c>
       <c r="B23" s="10">
-        <f>COUNTIF('Test Cases'!B2:B44,A23)</f>
+        <f>COUNTIF('Test Cases'!B2:B50,A23)</f>
         <v/>
       </c>
       <c r="C23" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B44,A23,'Test Cases'!G2:G44,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!B2:B50,A23,'Test Cases'!G2:G50,"Pass")</f>
         <v/>
       </c>
       <c r="D23" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B44,A23,'Test Cases'!G2:G44,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!B2:B50,A23,'Test Cases'!G2:G50,"Fail")</f>
         <v/>
       </c>
       <c r="E23" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B44,A23,'Test Cases'!G2:G44,"Not Run")</f>
+        <f>COUNTIFS('Test Cases'!B2:B50,A23,'Test Cases'!G2:G50,"Not Run")</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="14" t="inlineStr">
         <is>
+          <t>Fixed Assets</t>
+        </is>
+      </c>
+      <c r="B24" s="10">
+        <f>COUNTIF('Test Cases'!B2:B50,A24)</f>
+        <v/>
+      </c>
+      <c r="C24" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B50,A24,'Test Cases'!G2:G50,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D24" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B50,A24,'Test Cases'!G2:G50,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E24" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B50,A24,'Test Cases'!G2:G50,"Not Run")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="14" t="inlineStr">
+        <is>
           <t>End-to-End</t>
         </is>
       </c>
-      <c r="B24" s="10">
-        <f>COUNTIF('Test Cases'!B2:B44,A24)</f>
-        <v/>
-      </c>
-      <c r="C24" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B44,A24,'Test Cases'!G2:G44,"Pass")</f>
-        <v/>
-      </c>
-      <c r="D24" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B44,A24,'Test Cases'!G2:G44,"Fail")</f>
-        <v/>
-      </c>
-      <c r="E24" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B44,A24,'Test Cases'!G2:G44,"Not Run")</f>
+      <c r="B25" s="10">
+        <f>COUNTIF('Test Cases'!B2:B50,A25)</f>
+        <v/>
+      </c>
+      <c r="C25" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B50,A25,'Test Cases'!G2:G50,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D25" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B50,A25,'Test Cases'!G2:G50,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E25" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B50,A25,'Test Cases'!G2:G50,"Not Run")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: tambah Blueprint instalasi+konfigurasi & sinkronkan User Guide/UAT untuk 26 modul
- Blueprint_Installation_Configuration.docx (baru): arsitektur, katalog 26 modul,
  arsitektur data/integrasi, manual instalasi + urutan dependency, konfigurasi sistem
  (accounting/property, produk layanan, cron, CORETAX, portal/email), keamanan,
  alur E2E, pemeliharaan/backup.
- User Guide: overview diperluas ke 26 modul + section untuk document_ce, owner_portal,
  cam, rent_escalation, dashboard, dunning, insurance, lease_expiry, vacancy, ppm,
  parking, valuation, access, esign; catatan budget approval & multi-currency remittance.
- UAT Tracker: 79 test case mencakup seluruh modul baru.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016VgZWku95cicE6VZPkFTLL
</commit_message>
<xml_diff>
--- a/docs/UAT_Tracker_Custom_Modules.xlsx
+++ b/docs/UAT_Tracker_Custom_Modules.xlsx
@@ -530,7 +530,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J50"/>
+  <dimension ref="A1:J80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2360,32 +2360,32 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>E2E-1</t>
+          <t>DC-01</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>End-to-End</t>
+          <t>Documents CE</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Onboarding tenant</t>
+          <t>Unggah lampiran</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>Lead → Create Lease Contract → aktifkan → Handover Move-in → Guarantee.</t>
+          <t>Lampirkan 2 dokumen pada properti via tab Documents.</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>Kontrak aktif; handover selesai; jaminan Active; tenant bisa login portal.</t>
+          <t>documents_count=2; tersimpan sebagai ir.attachment milik properti.</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -2400,27 +2400,27 @@
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>E2E-2</t>
+          <t>OP-01</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>End-to-End</t>
+          <t>Owner Portal</t>
         </is>
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>Billing bulanan</t>
+          <t>Akses pemilik</t>
         </is>
       </c>
       <c r="D47" s="7" t="inlineStr">
         <is>
-          <t>Invoice sewa + Meter recharge + GTO turnover diposting.</t>
+          <t>Login sebagai owner portal yang memiliki properti.</t>
         </is>
       </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
-          <t>Semua pendapatan ber-link properti &amp; analytic; muncul di Owners Statement.</t>
+          <t>Daftar Properties hanya menampilkan properti miliknya.</t>
         </is>
       </c>
       <c r="F47" s="5" t="inlineStr">
@@ -2440,27 +2440,27 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>E2E-3</t>
+          <t>OP-02</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>End-to-End</t>
+          <t>Owner Portal</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>Pengeluaran</t>
+          <t>Isolasi data</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>Maintenance → Create PO → terima → vendor bill posted.</t>
+          <t>Owner A coba akses properti owner B via id URL.</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>Beban masuk Payment Details &amp; analytic properti.</t>
+          <t>Akses ditolak / diarahkan ke /my.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -2480,32 +2480,32 @@
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>E2E-4</t>
+          <t>OP-03</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>End-to-End</t>
+          <t>Owner Portal</t>
         </is>
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>Tutup periode</t>
+          <t>Lihat remittance</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>Cetak Owners Statement; Owner Remittance; ekspor CORETAX Faktur PK.</t>
+          <t>Buka detail properti dengan remittance posted.</t>
         </is>
       </c>
       <c r="E49" s="7" t="inlineStr">
         <is>
-          <t>Laporan konsisten; remittance terposting; XML e-Faktur terunduh.</t>
+          <t>Daftar remittance tampil dengan jumlah benar.</t>
         </is>
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G49" s="5" t="inlineStr">
@@ -2520,32 +2520,32 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>E2E-5</t>
+          <t>CM-01</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>End-to-End</t>
+          <t>CAM / Service Charge</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>Move-out</t>
+          <t>Apportion per area</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>Handover Move-out + make-good; Security Deposit refund; kontrak ditutup.</t>
+          <t>Pool=120jt; 3 tenant area 100/200/300 m². Apportion.</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>Deposit terselesaikan; Sec Dep Bal nol; kontrak closed.</t>
+          <t>Alokasi 20/40/60 jt sesuai proporsi area.</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -2557,9 +2557,1209 @@
       <c r="I50" s="2" t="inlineStr"/>
       <c r="J50" s="4" t="inlineStr"/>
     </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>CM-02</t>
+        </is>
+      </c>
+      <c r="B51" s="6" t="inlineStr">
+        <is>
+          <t>CAM / Service Charge</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="inlineStr">
+        <is>
+          <t>Invoice service charge</t>
+        </is>
+      </c>
+      <c r="D51" s="7" t="inlineStr">
+        <is>
+          <t>Klik Create Invoices.</t>
+        </is>
+      </c>
+      <c r="E51" s="7" t="inlineStr">
+        <is>
+          <t>out_invoice per tenant ber-link properti; muncul di Owners Statement &amp; analytic.</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G51" s="5" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="H51" s="6" t="inlineStr"/>
+      <c r="I51" s="5" t="inlineStr"/>
+      <c r="J51" s="7" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>CM-03</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>CAM / Service Charge</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>Budget vs actual</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>Isi actual berbeda dari budget.</t>
+        </is>
+      </c>
+      <c r="E52" s="4" t="inlineStr">
+        <is>
+          <t>Variance terhitung untuk rekonsiliasi.</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="inlineStr"/>
+      <c r="I52" s="2" t="inlineStr"/>
+      <c r="J52" s="4" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>RE-01</t>
+        </is>
+      </c>
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t>Rent Escalation</t>
+        </is>
+      </c>
+      <c r="C53" s="7" t="inlineStr">
+        <is>
+          <t>Eskalasi %</t>
+        </is>
+      </c>
+      <c r="D53" s="7" t="inlineStr">
+        <is>
+          <t>Sewa 10jt, 10%/tahun, due hari ini. Jalankan cron.</t>
+        </is>
+      </c>
+      <c r="E53" s="7" t="inlineStr">
+        <is>
+          <t>Sewa naik ke 11jt; log mencatat 10jt→11jt.</t>
+        </is>
+      </c>
+      <c r="F53" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G53" s="5" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="H53" s="6" t="inlineStr"/>
+      <c r="I53" s="5" t="inlineStr"/>
+      <c r="J53" s="7" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>RE-02</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>Rent Escalation</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>Eskalasi amount</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>Escalation +500rb. Jalankan cron.</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="inlineStr">
+        <is>
+          <t>Sewa naik 500rb; log tercatat.</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="inlineStr"/>
+      <c r="I54" s="2" t="inlineStr"/>
+      <c r="J54" s="4" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>RE-03</t>
+        </is>
+      </c>
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>Rent Escalation</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="inlineStr">
+        <is>
+          <t>Belum jatuh tempo</t>
+        </is>
+      </c>
+      <c r="D55" s="7" t="inlineStr">
+        <is>
+          <t>Tanggal due di masa depan. Jalankan cron.</t>
+        </is>
+      </c>
+      <c r="E55" s="7" t="inlineStr">
+        <is>
+          <t>Tidak ada perubahan sewa.</t>
+        </is>
+      </c>
+      <c r="F55" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G55" s="5" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="H55" s="6" t="inlineStr"/>
+      <c r="I55" s="5" t="inlineStr"/>
+      <c r="J55" s="7" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>DB-01</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>KPI Dashboard</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>Hitung KPI</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>Dengan kontrak &amp; invoice ada, buka Dashboard.</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="inlineStr">
+        <is>
+          <t>NOI=income−expense; arrears=invoice overdue; collection rate konsisten.</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="H56" s="3" t="inlineStr"/>
+      <c r="I56" s="2" t="inlineStr"/>
+      <c r="J56" s="4" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>DB-02</t>
+        </is>
+      </c>
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>KPI Dashboard</t>
+        </is>
+      </c>
+      <c r="C57" s="7" t="inlineStr">
+        <is>
+          <t>Lease expiring</t>
+        </is>
+      </c>
+      <c r="D57" s="7" t="inlineStr">
+        <is>
+          <t>Ada kontrak berakhir dalam 12 bulan.</t>
+        </is>
+      </c>
+      <c r="E57" s="7" t="inlineStr">
+        <is>
+          <t>Counter leases-expiring menampilkan jumlah benar.</t>
+        </is>
+      </c>
+      <c r="F57" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G57" s="5" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="H57" s="6" t="inlineStr"/>
+      <c r="I57" s="5" t="inlineStr"/>
+      <c r="J57" s="7" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>DN-01</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>Dunning</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>Naik level</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>Invoice overdue melewati ambang level 1. Jalankan cron.</t>
+        </is>
+      </c>
+      <c r="E58" s="4" t="inlineStr">
+        <is>
+          <t>Dunning level=1; email reminder terkirim.</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="inlineStr"/>
+      <c r="I58" s="2" t="inlineStr"/>
+      <c r="J58" s="4" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr">
+        <is>
+          <t>DN-02</t>
+        </is>
+      </c>
+      <c r="B59" s="6" t="inlineStr">
+        <is>
+          <t>Dunning</t>
+        </is>
+      </c>
+      <c r="C59" s="7" t="inlineStr">
+        <is>
+          <t>Late fee</t>
+        </is>
+      </c>
+      <c r="D59" s="7" t="inlineStr">
+        <is>
+          <t>Aktifkan late fee pada level. Jalankan cron.</t>
+        </is>
+      </c>
+      <c r="E59" s="7" t="inlineStr">
+        <is>
+          <t>Denda ditambahkan sesuai konfigurasi.</t>
+        </is>
+      </c>
+      <c r="F59" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G59" s="5" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="H59" s="6" t="inlineStr"/>
+      <c r="I59" s="5" t="inlineStr"/>
+      <c r="J59" s="7" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>DN-03</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>Dunning</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>Lunas berhenti</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="inlineStr">
+        <is>
+          <t>Bayar invoice. Jalankan cron.</t>
+        </is>
+      </c>
+      <c r="E60" s="4" t="inlineStr">
+        <is>
+          <t>Tidak ada reminder lanjutan.</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="H60" s="3" t="inlineStr"/>
+      <c r="I60" s="2" t="inlineStr"/>
+      <c r="J60" s="4" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
+        <is>
+          <t>IN-01</t>
+        </is>
+      </c>
+      <c r="B61" s="6" t="inlineStr">
+        <is>
+          <t>Insurance</t>
+        </is>
+      </c>
+      <c r="C61" s="7" t="inlineStr">
+        <is>
+          <t>Buat polis</t>
+        </is>
+      </c>
+      <c r="D61" s="7" t="inlineStr">
+        <is>
+          <t>Buat polis expiry 30 hari ke depan.</t>
+        </is>
+      </c>
+      <c r="E61" s="7" t="inlineStr">
+        <is>
+          <t>Polis tersimpan; days-to-expiry terhitung.</t>
+        </is>
+      </c>
+      <c r="F61" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G61" s="5" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="H61" s="6" t="inlineStr"/>
+      <c r="I61" s="5" t="inlineStr"/>
+      <c r="J61" s="7" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>IN-02</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>Insurance</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t>Reminder</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>Expiry dalam lead window. Jalankan cron.</t>
+        </is>
+      </c>
+      <c r="E62" s="4" t="inlineStr">
+        <is>
+          <t>Activity reminder terjadwal pada penanggung jawab.</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="H62" s="3" t="inlineStr"/>
+      <c r="I62" s="2" t="inlineStr"/>
+      <c r="J62" s="4" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr">
+        <is>
+          <t>LE-01</t>
+        </is>
+      </c>
+      <c r="B63" s="6" t="inlineStr">
+        <is>
+          <t>Lease Expiry</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
+          <t>Filter 30 hari</t>
+        </is>
+      </c>
+      <c r="D63" s="7" t="inlineStr">
+        <is>
+          <t>Kontrak berakhir dalam 20 hari.</t>
+        </is>
+      </c>
+      <c r="E63" s="7" t="inlineStr">
+        <is>
+          <t>Muncul pada filter 30 hari.</t>
+        </is>
+      </c>
+      <c r="F63" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G63" s="5" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="H63" s="6" t="inlineStr"/>
+      <c r="I63" s="5" t="inlineStr"/>
+      <c r="J63" s="7" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>LE-02</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>Lease Expiry</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
+        <is>
+          <t>Reminder renewal</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t>Jalankan cron.</t>
+        </is>
+      </c>
+      <c r="E64" s="4" t="inlineStr">
+        <is>
+          <t>Activity reminder renewal terjadwal.</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="H64" s="3" t="inlineStr"/>
+      <c r="I64" s="2" t="inlineStr"/>
+      <c r="J64" s="4" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr">
+        <is>
+          <t>VC-01</t>
+        </is>
+      </c>
+      <c r="B65" s="6" t="inlineStr">
+        <is>
+          <t>Vacancy</t>
+        </is>
+      </c>
+      <c r="C65" s="7" t="inlineStr">
+        <is>
+          <t>Kelompok status</t>
+        </is>
+      </c>
+      <c r="D65" s="7" t="inlineStr">
+        <is>
+          <t>Beberapa properti status berbeda.</t>
+        </is>
+      </c>
+      <c r="E65" s="7" t="inlineStr">
+        <is>
+          <t>Board mengelompokkan benar sesuai stage.</t>
+        </is>
+      </c>
+      <c r="F65" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G65" s="5" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="H65" s="6" t="inlineStr"/>
+      <c r="I65" s="5" t="inlineStr"/>
+      <c r="J65" s="7" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>VC-02</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>Vacancy</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>Filter available</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>Pilih filter Available.</t>
+        </is>
+      </c>
+      <c r="E66" s="4" t="inlineStr">
+        <is>
+          <t>Hanya properti available tampil.</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="H66" s="3" t="inlineStr"/>
+      <c r="I66" s="2" t="inlineStr"/>
+      <c r="J66" s="4" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="inlineStr">
+        <is>
+          <t>PP-01</t>
+        </is>
+      </c>
+      <c r="B67" s="6" t="inlineStr">
+        <is>
+          <t>PPM</t>
+        </is>
+      </c>
+      <c r="C67" s="7" t="inlineStr">
+        <is>
+          <t>Generate request</t>
+        </is>
+      </c>
+      <c r="D67" s="7" t="inlineStr">
+        <is>
+          <t>PPM plan due hari ini. Jalankan cron.</t>
+        </is>
+      </c>
+      <c r="E67" s="7" t="inlineStr">
+        <is>
+          <t>maintenance.request baru terbuat sesuai plan.</t>
+        </is>
+      </c>
+      <c r="F67" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G67" s="5" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="H67" s="6" t="inlineStr"/>
+      <c r="I67" s="5" t="inlineStr"/>
+      <c r="J67" s="7" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>PP-02</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>PPM</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t>Interval berikut</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>Setelah generate, cek next date.</t>
+        </is>
+      </c>
+      <c r="E68" s="4" t="inlineStr">
+        <is>
+          <t>Tanggal jadwal berikut bergeser sesuai interval.</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="H68" s="3" t="inlineStr"/>
+      <c r="I68" s="2" t="inlineStr"/>
+      <c r="J68" s="4" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="5" t="inlineStr">
+        <is>
+          <t>PK-01</t>
+        </is>
+      </c>
+      <c r="B69" s="6" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="C69" s="7" t="inlineStr">
+        <is>
+          <t>Alokasi bay</t>
+        </is>
+      </c>
+      <c r="D69" s="7" t="inlineStr">
+        <is>
+          <t>Tetapkan bay ke tenant.</t>
+        </is>
+      </c>
+      <c r="E69" s="7" t="inlineStr">
+        <is>
+          <t>Bay berstatus allocated; terkait tenant/kontrak.</t>
+        </is>
+      </c>
+      <c r="F69" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G69" s="5" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="H69" s="6" t="inlineStr"/>
+      <c r="I69" s="5" t="inlineStr"/>
+      <c r="J69" s="7" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>PK-02</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t>Invoice parkir</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr">
+        <is>
+          <t>Buat invoice parkir.</t>
+        </is>
+      </c>
+      <c r="E70" s="4" t="inlineStr">
+        <is>
+          <t>out_invoice ber-link properti; muncul di Owners Statement.</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="H70" s="3" t="inlineStr"/>
+      <c r="I70" s="2" t="inlineStr"/>
+      <c r="J70" s="4" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="5" t="inlineStr">
+        <is>
+          <t>VL-01</t>
+        </is>
+      </c>
+      <c r="B71" s="6" t="inlineStr">
+        <is>
+          <t>Valuation</t>
+        </is>
+      </c>
+      <c r="C71" s="7" t="inlineStr">
+        <is>
+          <t>Catat valuasi</t>
+        </is>
+      </c>
+      <c r="D71" s="7" t="inlineStr">
+        <is>
+          <t>Buat 2 valuasi tanggal berbeda.</t>
+        </is>
+      </c>
+      <c r="E71" s="7" t="inlineStr">
+        <is>
+          <t>Latest value = valuasi tanggal terbaru.</t>
+        </is>
+      </c>
+      <c r="F71" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G71" s="5" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="H71" s="6" t="inlineStr"/>
+      <c r="I71" s="5" t="inlineStr"/>
+      <c r="J71" s="7" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>AC-01</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>Access</t>
+        </is>
+      </c>
+      <c r="C72" s="4" t="inlineStr">
+        <is>
+          <t>Terbitkan kartu</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="inlineStr">
+        <is>
+          <t>Buat kartu akses untuk tenant.</t>
+        </is>
+      </c>
+      <c r="E72" s="4" t="inlineStr">
+        <is>
+          <t>Kartu tercatat &amp; terkait tenant.</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="H72" s="3" t="inlineStr"/>
+      <c r="I72" s="2" t="inlineStr"/>
+      <c r="J72" s="4" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="5" t="inlineStr">
+        <is>
+          <t>AC-02</t>
+        </is>
+      </c>
+      <c r="B73" s="6" t="inlineStr">
+        <is>
+          <t>Access</t>
+        </is>
+      </c>
+      <c r="C73" s="7" t="inlineStr">
+        <is>
+          <t>Log tamu</t>
+        </is>
+      </c>
+      <c r="D73" s="7" t="inlineStr">
+        <is>
+          <t>Catat check-in lalu check-out tamu.</t>
+        </is>
+      </c>
+      <c r="E73" s="7" t="inlineStr">
+        <is>
+          <t>Waktu check-in/out tersimpan.</t>
+        </is>
+      </c>
+      <c r="F73" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G73" s="5" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="H73" s="6" t="inlineStr"/>
+      <c r="I73" s="5" t="inlineStr"/>
+      <c r="J73" s="7" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>ES-01</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>E-Signature</t>
+        </is>
+      </c>
+      <c r="C74" s="4" t="inlineStr">
+        <is>
+          <t>Kirim permintaan</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="inlineStr">
+        <is>
+          <t>Klik Request Signature pada kontrak.</t>
+        </is>
+      </c>
+      <c r="E74" s="4" t="inlineStr">
+        <is>
+          <t>Status=Sent; sequence terbuat; email/log tercatat.</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="H74" s="3" t="inlineStr"/>
+      <c r="I74" s="2" t="inlineStr"/>
+      <c r="J74" s="4" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="5" t="inlineStr">
+        <is>
+          <t>ES-02</t>
+        </is>
+      </c>
+      <c r="B75" s="6" t="inlineStr">
+        <is>
+          <t>E-Signature</t>
+        </is>
+      </c>
+      <c r="C75" s="7" t="inlineStr">
+        <is>
+          <t>Tandai signed</t>
+        </is>
+      </c>
+      <c r="D75" s="7" t="inlineStr">
+        <is>
+          <t>Klik Mark Signed.</t>
+        </is>
+      </c>
+      <c r="E75" s="7" t="inlineStr">
+        <is>
+          <t>Status=Signed; tanggal tanda tangan tersimpan.</t>
+        </is>
+      </c>
+      <c r="F75" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G75" s="5" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="H75" s="6" t="inlineStr"/>
+      <c r="I75" s="5" t="inlineStr"/>
+      <c r="J75" s="7" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>E2E-1</t>
+        </is>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>End-to-End</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="inlineStr">
+        <is>
+          <t>Onboarding tenant</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="inlineStr">
+        <is>
+          <t>Lead → Create Lease Contract → aktifkan → Handover Move-in → Guarantee.</t>
+        </is>
+      </c>
+      <c r="E76" s="4" t="inlineStr">
+        <is>
+          <t>Kontrak aktif; handover selesai; jaminan Active; tenant bisa login portal.</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="H76" s="3" t="inlineStr"/>
+      <c r="I76" s="2" t="inlineStr"/>
+      <c r="J76" s="4" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="5" t="inlineStr">
+        <is>
+          <t>E2E-2</t>
+        </is>
+      </c>
+      <c r="B77" s="6" t="inlineStr">
+        <is>
+          <t>End-to-End</t>
+        </is>
+      </c>
+      <c r="C77" s="7" t="inlineStr">
+        <is>
+          <t>Billing bulanan</t>
+        </is>
+      </c>
+      <c r="D77" s="7" t="inlineStr">
+        <is>
+          <t>Invoice sewa + Meter recharge + GTO turnover diposting.</t>
+        </is>
+      </c>
+      <c r="E77" s="7" t="inlineStr">
+        <is>
+          <t>Semua pendapatan ber-link properti &amp; analytic; muncul di Owners Statement.</t>
+        </is>
+      </c>
+      <c r="F77" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G77" s="5" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="H77" s="6" t="inlineStr"/>
+      <c r="I77" s="5" t="inlineStr"/>
+      <c r="J77" s="7" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>E2E-3</t>
+        </is>
+      </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>End-to-End</t>
+        </is>
+      </c>
+      <c r="C78" s="4" t="inlineStr">
+        <is>
+          <t>Pengeluaran</t>
+        </is>
+      </c>
+      <c r="D78" s="4" t="inlineStr">
+        <is>
+          <t>Maintenance → Create PO → terima → vendor bill posted.</t>
+        </is>
+      </c>
+      <c r="E78" s="4" t="inlineStr">
+        <is>
+          <t>Beban masuk Payment Details &amp; analytic properti.</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="H78" s="3" t="inlineStr"/>
+      <c r="I78" s="2" t="inlineStr"/>
+      <c r="J78" s="4" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="5" t="inlineStr">
+        <is>
+          <t>E2E-4</t>
+        </is>
+      </c>
+      <c r="B79" s="6" t="inlineStr">
+        <is>
+          <t>End-to-End</t>
+        </is>
+      </c>
+      <c r="C79" s="7" t="inlineStr">
+        <is>
+          <t>Tutup periode</t>
+        </is>
+      </c>
+      <c r="D79" s="7" t="inlineStr">
+        <is>
+          <t>Cetak Owners Statement; Owner Remittance; ekspor CORETAX Faktur PK.</t>
+        </is>
+      </c>
+      <c r="E79" s="7" t="inlineStr">
+        <is>
+          <t>Laporan konsisten; remittance terposting; XML e-Faktur terunduh.</t>
+        </is>
+      </c>
+      <c r="F79" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G79" s="5" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="H79" s="6" t="inlineStr"/>
+      <c r="I79" s="5" t="inlineStr"/>
+      <c r="J79" s="7" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>E2E-5</t>
+        </is>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>End-to-End</t>
+        </is>
+      </c>
+      <c r="C80" s="4" t="inlineStr">
+        <is>
+          <t>Move-out</t>
+        </is>
+      </c>
+      <c r="D80" s="4" t="inlineStr">
+        <is>
+          <t>Handover Move-out + make-good; Security Deposit refund; kontrak ditutup.</t>
+        </is>
+      </c>
+      <c r="E80" s="4" t="inlineStr">
+        <is>
+          <t>Deposit terselesaikan; Sec Dep Bal nol; kontrak closed.</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="H80" s="3" t="inlineStr"/>
+      <c r="I80" s="2" t="inlineStr"/>
+      <c r="J80" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
-  <conditionalFormatting sqref="G2:G50">
+  <conditionalFormatting sqref="G2:G80">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -2574,10 +3774,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="G2:G50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G2:G80" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not Run,Pass,Fail,Blocked,N/A"</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F80" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"High,Medium,Low"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2591,7 +3791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2615,7 +3815,7 @@
         </is>
       </c>
       <c r="B3" s="10">
-        <f>COUNTA('Test Cases'!A2:A50)</f>
+        <f>COUNTA('Test Cases'!A2:A80)</f>
         <v/>
       </c>
     </row>
@@ -2626,7 +3826,7 @@
         </is>
       </c>
       <c r="B4" s="10">
-        <f>COUNTIF('Test Cases'!G2:G50,"Pass")</f>
+        <f>COUNTIF('Test Cases'!G2:G80,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -2637,7 +3837,7 @@
         </is>
       </c>
       <c r="B5" s="10">
-        <f>COUNTIF('Test Cases'!G2:G50,"Fail")</f>
+        <f>COUNTIF('Test Cases'!G2:G80,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -2648,7 +3848,7 @@
         </is>
       </c>
       <c r="B6" s="10">
-        <f>COUNTIF('Test Cases'!G2:G50,"Blocked")</f>
+        <f>COUNTIF('Test Cases'!G2:G80,"Blocked")</f>
         <v/>
       </c>
     </row>
@@ -2659,7 +3859,7 @@
         </is>
       </c>
       <c r="B7" s="10">
-        <f>COUNTIF('Test Cases'!G2:G50,"N/A")</f>
+        <f>COUNTIF('Test Cases'!G2:G80,"N/A")</f>
         <v/>
       </c>
     </row>
@@ -2670,7 +3870,7 @@
         </is>
       </c>
       <c r="B8" s="10">
-        <f>COUNTIF('Test Cases'!G2:G50,"Not Run")</f>
+        <f>COUNTIF('Test Cases'!G2:G80,"Not Run")</f>
         <v/>
       </c>
     </row>
@@ -2726,19 +3926,19 @@
         </is>
       </c>
       <c r="B13" s="10">
-        <f>COUNTIF('Test Cases'!B2:B50,A13)</f>
+        <f>COUNTIF('Test Cases'!B2:B80,A13)</f>
         <v/>
       </c>
       <c r="C13" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B50,A13,'Test Cases'!G2:G50,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!B2:B80,A13,'Test Cases'!G2:G80,"Pass")</f>
         <v/>
       </c>
       <c r="D13" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B50,A13,'Test Cases'!G2:G50,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!B2:B80,A13,'Test Cases'!G2:G80,"Fail")</f>
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B50,A13,'Test Cases'!G2:G50,"Not Run")</f>
+        <f>COUNTIFS('Test Cases'!B2:B80,A13,'Test Cases'!G2:G80,"Not Run")</f>
         <v/>
       </c>
     </row>
@@ -2749,19 +3949,19 @@
         </is>
       </c>
       <c r="B14" s="10">
-        <f>COUNTIF('Test Cases'!B2:B50,A14)</f>
+        <f>COUNTIF('Test Cases'!B2:B80,A14)</f>
         <v/>
       </c>
       <c r="C14" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B50,A14,'Test Cases'!G2:G50,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!B2:B80,A14,'Test Cases'!G2:G80,"Pass")</f>
         <v/>
       </c>
       <c r="D14" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B50,A14,'Test Cases'!G2:G50,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!B2:B80,A14,'Test Cases'!G2:G80,"Fail")</f>
         <v/>
       </c>
       <c r="E14" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B50,A14,'Test Cases'!G2:G50,"Not Run")</f>
+        <f>COUNTIFS('Test Cases'!B2:B80,A14,'Test Cases'!G2:G80,"Not Run")</f>
         <v/>
       </c>
     </row>
@@ -2772,19 +3972,19 @@
         </is>
       </c>
       <c r="B15" s="10">
-        <f>COUNTIF('Test Cases'!B2:B50,A15)</f>
+        <f>COUNTIF('Test Cases'!B2:B80,A15)</f>
         <v/>
       </c>
       <c r="C15" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B50,A15,'Test Cases'!G2:G50,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!B2:B80,A15,'Test Cases'!G2:G80,"Pass")</f>
         <v/>
       </c>
       <c r="D15" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B50,A15,'Test Cases'!G2:G50,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!B2:B80,A15,'Test Cases'!G2:G80,"Fail")</f>
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B50,A15,'Test Cases'!G2:G50,"Not Run")</f>
+        <f>COUNTIFS('Test Cases'!B2:B80,A15,'Test Cases'!G2:G80,"Not Run")</f>
         <v/>
       </c>
     </row>
@@ -2795,19 +3995,19 @@
         </is>
       </c>
       <c r="B16" s="10">
-        <f>COUNTIF('Test Cases'!B2:B50,A16)</f>
+        <f>COUNTIF('Test Cases'!B2:B80,A16)</f>
         <v/>
       </c>
       <c r="C16" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B50,A16,'Test Cases'!G2:G50,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!B2:B80,A16,'Test Cases'!G2:G80,"Pass")</f>
         <v/>
       </c>
       <c r="D16" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B50,A16,'Test Cases'!G2:G50,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!B2:B80,A16,'Test Cases'!G2:G80,"Fail")</f>
         <v/>
       </c>
       <c r="E16" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B50,A16,'Test Cases'!G2:G50,"Not Run")</f>
+        <f>COUNTIFS('Test Cases'!B2:B80,A16,'Test Cases'!G2:G80,"Not Run")</f>
         <v/>
       </c>
     </row>
@@ -2818,19 +4018,19 @@
         </is>
       </c>
       <c r="B17" s="10">
-        <f>COUNTIF('Test Cases'!B2:B50,A17)</f>
+        <f>COUNTIF('Test Cases'!B2:B80,A17)</f>
         <v/>
       </c>
       <c r="C17" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B50,A17,'Test Cases'!G2:G50,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!B2:B80,A17,'Test Cases'!G2:G80,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B50,A17,'Test Cases'!G2:G50,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!B2:B80,A17,'Test Cases'!G2:G80,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B50,A17,'Test Cases'!G2:G50,"Not Run")</f>
+        <f>COUNTIFS('Test Cases'!B2:B80,A17,'Test Cases'!G2:G80,"Not Run")</f>
         <v/>
       </c>
     </row>
@@ -2841,19 +4041,19 @@
         </is>
       </c>
       <c r="B18" s="10">
-        <f>COUNTIF('Test Cases'!B2:B50,A18)</f>
+        <f>COUNTIF('Test Cases'!B2:B80,A18)</f>
         <v/>
       </c>
       <c r="C18" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B50,A18,'Test Cases'!G2:G50,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!B2:B80,A18,'Test Cases'!G2:G80,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B50,A18,'Test Cases'!G2:G50,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!B2:B80,A18,'Test Cases'!G2:G80,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B50,A18,'Test Cases'!G2:G50,"Not Run")</f>
+        <f>COUNTIFS('Test Cases'!B2:B80,A18,'Test Cases'!G2:G80,"Not Run")</f>
         <v/>
       </c>
     </row>
@@ -2864,19 +4064,19 @@
         </is>
       </c>
       <c r="B19" s="10">
-        <f>COUNTIF('Test Cases'!B2:B50,A19)</f>
+        <f>COUNTIF('Test Cases'!B2:B80,A19)</f>
         <v/>
       </c>
       <c r="C19" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B50,A19,'Test Cases'!G2:G50,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!B2:B80,A19,'Test Cases'!G2:G80,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B50,A19,'Test Cases'!G2:G50,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!B2:B80,A19,'Test Cases'!G2:G80,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B50,A19,'Test Cases'!G2:G50,"Not Run")</f>
+        <f>COUNTIFS('Test Cases'!B2:B80,A19,'Test Cases'!G2:G80,"Not Run")</f>
         <v/>
       </c>
     </row>
@@ -2887,19 +4087,19 @@
         </is>
       </c>
       <c r="B20" s="10">
-        <f>COUNTIF('Test Cases'!B2:B50,A20)</f>
+        <f>COUNTIF('Test Cases'!B2:B80,A20)</f>
         <v/>
       </c>
       <c r="C20" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B50,A20,'Test Cases'!G2:G50,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!B2:B80,A20,'Test Cases'!G2:G80,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B50,A20,'Test Cases'!G2:G50,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!B2:B80,A20,'Test Cases'!G2:G80,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B50,A20,'Test Cases'!G2:G50,"Not Run")</f>
+        <f>COUNTIFS('Test Cases'!B2:B80,A20,'Test Cases'!G2:G80,"Not Run")</f>
         <v/>
       </c>
     </row>
@@ -2910,19 +4110,19 @@
         </is>
       </c>
       <c r="B21" s="10">
-        <f>COUNTIF('Test Cases'!B2:B50,A21)</f>
+        <f>COUNTIF('Test Cases'!B2:B80,A21)</f>
         <v/>
       </c>
       <c r="C21" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B50,A21,'Test Cases'!G2:G50,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!B2:B80,A21,'Test Cases'!G2:G80,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B50,A21,'Test Cases'!G2:G50,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!B2:B80,A21,'Test Cases'!G2:G80,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B50,A21,'Test Cases'!G2:G50,"Not Run")</f>
+        <f>COUNTIFS('Test Cases'!B2:B80,A21,'Test Cases'!G2:G80,"Not Run")</f>
         <v/>
       </c>
     </row>
@@ -2933,19 +4133,19 @@
         </is>
       </c>
       <c r="B22" s="10">
-        <f>COUNTIF('Test Cases'!B2:B50,A22)</f>
+        <f>COUNTIF('Test Cases'!B2:B80,A22)</f>
         <v/>
       </c>
       <c r="C22" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B50,A22,'Test Cases'!G2:G50,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!B2:B80,A22,'Test Cases'!G2:G80,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B50,A22,'Test Cases'!G2:G50,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!B2:B80,A22,'Test Cases'!G2:G80,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B50,A22,'Test Cases'!G2:G50,"Not Run")</f>
+        <f>COUNTIFS('Test Cases'!B2:B80,A22,'Test Cases'!G2:G80,"Not Run")</f>
         <v/>
       </c>
     </row>
@@ -2956,19 +4156,19 @@
         </is>
       </c>
       <c r="B23" s="10">
-        <f>COUNTIF('Test Cases'!B2:B50,A23)</f>
+        <f>COUNTIF('Test Cases'!B2:B80,A23)</f>
         <v/>
       </c>
       <c r="C23" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B50,A23,'Test Cases'!G2:G50,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!B2:B80,A23,'Test Cases'!G2:G80,"Pass")</f>
         <v/>
       </c>
       <c r="D23" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B50,A23,'Test Cases'!G2:G50,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!B2:B80,A23,'Test Cases'!G2:G80,"Fail")</f>
         <v/>
       </c>
       <c r="E23" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B50,A23,'Test Cases'!G2:G50,"Not Run")</f>
+        <f>COUNTIFS('Test Cases'!B2:B80,A23,'Test Cases'!G2:G80,"Not Run")</f>
         <v/>
       </c>
     </row>
@@ -2979,42 +4179,364 @@
         </is>
       </c>
       <c r="B24" s="10">
-        <f>COUNTIF('Test Cases'!B2:B50,A24)</f>
+        <f>COUNTIF('Test Cases'!B2:B80,A24)</f>
         <v/>
       </c>
       <c r="C24" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B50,A24,'Test Cases'!G2:G50,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!B2:B80,A24,'Test Cases'!G2:G80,"Pass")</f>
         <v/>
       </c>
       <c r="D24" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B50,A24,'Test Cases'!G2:G50,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!B2:B80,A24,'Test Cases'!G2:G80,"Fail")</f>
         <v/>
       </c>
       <c r="E24" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B50,A24,'Test Cases'!G2:G50,"Not Run")</f>
+        <f>COUNTIFS('Test Cases'!B2:B80,A24,'Test Cases'!G2:G80,"Not Run")</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="14" t="inlineStr">
         <is>
+          <t>Documents CE</t>
+        </is>
+      </c>
+      <c r="B25" s="10">
+        <f>COUNTIF('Test Cases'!B2:B80,A25)</f>
+        <v/>
+      </c>
+      <c r="C25" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A25,'Test Cases'!G2:G80,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D25" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A25,'Test Cases'!G2:G80,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E25" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A25,'Test Cases'!G2:G80,"Not Run")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="14" t="inlineStr">
+        <is>
+          <t>Owner Portal</t>
+        </is>
+      </c>
+      <c r="B26" s="10">
+        <f>COUNTIF('Test Cases'!B2:B80,A26)</f>
+        <v/>
+      </c>
+      <c r="C26" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A26,'Test Cases'!G2:G80,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D26" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A26,'Test Cases'!G2:G80,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E26" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A26,'Test Cases'!G2:G80,"Not Run")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="14" t="inlineStr">
+        <is>
+          <t>CAM / Service Charge</t>
+        </is>
+      </c>
+      <c r="B27" s="10">
+        <f>COUNTIF('Test Cases'!B2:B80,A27)</f>
+        <v/>
+      </c>
+      <c r="C27" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A27,'Test Cases'!G2:G80,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D27" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A27,'Test Cases'!G2:G80,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E27" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A27,'Test Cases'!G2:G80,"Not Run")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="14" t="inlineStr">
+        <is>
+          <t>Rent Escalation</t>
+        </is>
+      </c>
+      <c r="B28" s="10">
+        <f>COUNTIF('Test Cases'!B2:B80,A28)</f>
+        <v/>
+      </c>
+      <c r="C28" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A28,'Test Cases'!G2:G80,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D28" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A28,'Test Cases'!G2:G80,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E28" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A28,'Test Cases'!G2:G80,"Not Run")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="14" t="inlineStr">
+        <is>
+          <t>KPI Dashboard</t>
+        </is>
+      </c>
+      <c r="B29" s="10">
+        <f>COUNTIF('Test Cases'!B2:B80,A29)</f>
+        <v/>
+      </c>
+      <c r="C29" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A29,'Test Cases'!G2:G80,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D29" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A29,'Test Cases'!G2:G80,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E29" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A29,'Test Cases'!G2:G80,"Not Run")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="14" t="inlineStr">
+        <is>
+          <t>Dunning</t>
+        </is>
+      </c>
+      <c r="B30" s="10">
+        <f>COUNTIF('Test Cases'!B2:B80,A30)</f>
+        <v/>
+      </c>
+      <c r="C30" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A30,'Test Cases'!G2:G80,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D30" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A30,'Test Cases'!G2:G80,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E30" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A30,'Test Cases'!G2:G80,"Not Run")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="14" t="inlineStr">
+        <is>
+          <t>Insurance</t>
+        </is>
+      </c>
+      <c r="B31" s="10">
+        <f>COUNTIF('Test Cases'!B2:B80,A31)</f>
+        <v/>
+      </c>
+      <c r="C31" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A31,'Test Cases'!G2:G80,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D31" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A31,'Test Cases'!G2:G80,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E31" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A31,'Test Cases'!G2:G80,"Not Run")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="14" t="inlineStr">
+        <is>
+          <t>Lease Expiry</t>
+        </is>
+      </c>
+      <c r="B32" s="10">
+        <f>COUNTIF('Test Cases'!B2:B80,A32)</f>
+        <v/>
+      </c>
+      <c r="C32" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A32,'Test Cases'!G2:G80,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D32" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A32,'Test Cases'!G2:G80,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E32" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A32,'Test Cases'!G2:G80,"Not Run")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="14" t="inlineStr">
+        <is>
+          <t>Vacancy</t>
+        </is>
+      </c>
+      <c r="B33" s="10">
+        <f>COUNTIF('Test Cases'!B2:B80,A33)</f>
+        <v/>
+      </c>
+      <c r="C33" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A33,'Test Cases'!G2:G80,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D33" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A33,'Test Cases'!G2:G80,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E33" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A33,'Test Cases'!G2:G80,"Not Run")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="14" t="inlineStr">
+        <is>
+          <t>PPM</t>
+        </is>
+      </c>
+      <c r="B34" s="10">
+        <f>COUNTIF('Test Cases'!B2:B80,A34)</f>
+        <v/>
+      </c>
+      <c r="C34" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A34,'Test Cases'!G2:G80,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D34" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A34,'Test Cases'!G2:G80,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E34" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A34,'Test Cases'!G2:G80,"Not Run")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="14" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="B35" s="10">
+        <f>COUNTIF('Test Cases'!B2:B80,A35)</f>
+        <v/>
+      </c>
+      <c r="C35" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A35,'Test Cases'!G2:G80,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D35" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A35,'Test Cases'!G2:G80,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E35" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A35,'Test Cases'!G2:G80,"Not Run")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="14" t="inlineStr">
+        <is>
+          <t>Valuation</t>
+        </is>
+      </c>
+      <c r="B36" s="10">
+        <f>COUNTIF('Test Cases'!B2:B80,A36)</f>
+        <v/>
+      </c>
+      <c r="C36" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A36,'Test Cases'!G2:G80,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D36" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A36,'Test Cases'!G2:G80,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E36" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A36,'Test Cases'!G2:G80,"Not Run")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="14" t="inlineStr">
+        <is>
+          <t>Access</t>
+        </is>
+      </c>
+      <c r="B37" s="10">
+        <f>COUNTIF('Test Cases'!B2:B80,A37)</f>
+        <v/>
+      </c>
+      <c r="C37" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A37,'Test Cases'!G2:G80,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D37" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A37,'Test Cases'!G2:G80,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E37" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A37,'Test Cases'!G2:G80,"Not Run")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="14" t="inlineStr">
+        <is>
+          <t>E-Signature</t>
+        </is>
+      </c>
+      <c r="B38" s="10">
+        <f>COUNTIF('Test Cases'!B2:B80,A38)</f>
+        <v/>
+      </c>
+      <c r="C38" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A38,'Test Cases'!G2:G80,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D38" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A38,'Test Cases'!G2:G80,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E38" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A38,'Test Cases'!G2:G80,"Not Run")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="14" t="inlineStr">
+        <is>
           <t>End-to-End</t>
         </is>
       </c>
-      <c r="B25" s="10">
-        <f>COUNTIF('Test Cases'!B2:B50,A25)</f>
-        <v/>
-      </c>
-      <c r="C25" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B50,A25,'Test Cases'!G2:G50,"Pass")</f>
-        <v/>
-      </c>
-      <c r="D25" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B50,A25,'Test Cases'!G2:G50,"Fail")</f>
-        <v/>
-      </c>
-      <c r="E25" s="10">
-        <f>COUNTIFS('Test Cases'!B2:B50,A25,'Test Cases'!G2:G50,"Not Run")</f>
+      <c r="B39" s="10">
+        <f>COUNTIF('Test Cases'!B2:B80,A39)</f>
+        <v/>
+      </c>
+      <c r="C39" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A39,'Test Cases'!G2:G80,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D39" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A39,'Test Cases'!G2:G80,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E39" s="10">
+        <f>COUNTIFS('Test Cases'!B2:B80,A39,'Test Cases'!G2:G80,"Not Run")</f>
         <v/>
       </c>
     </row>

</xml_diff>